<commit_message>
Grass25 refactoring - fix stage code
</commit_message>
<xml_diff>
--- a/Tests/Validation/Wheat/UoM_WheatProject/GrassPatch2025_Observed.xlsx
+++ b/Tests/Validation/Wheat/UoM_WheatProject/GrassPatch2025_Observed.xlsx
@@ -1490,7 +1490,7 @@
         <v>45962</v>
       </c>
       <c r="AV34">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35">
@@ -2608,7 +2608,7 @@
         <v>45961</v>
       </c>
       <c r="AV74">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="75">
@@ -3651,7 +3651,7 @@
         <v>45961</v>
       </c>
       <c r="AV111">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="112">
@@ -4769,7 +4769,7 @@
         <v>45964</v>
       </c>
       <c r="AV151">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="152">
@@ -5743,7 +5743,7 @@
         <v>45956</v>
       </c>
       <c r="AV185">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="186">
@@ -6809,7 +6809,7 @@
         <v>45958</v>
       </c>
       <c r="AV223">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="224">
@@ -7927,7 +7927,7 @@
         <v>45959</v>
       </c>
       <c r="AV263">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="264">
@@ -9045,7 +9045,7 @@
         <v>45959</v>
       </c>
       <c r="AV303">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="304">
@@ -10186,7 +10186,7 @@
         <v>45962</v>
       </c>
       <c r="AV344">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="345">
@@ -11206,7 +11206,7 @@
         <v>45957</v>
       </c>
       <c r="AV380">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="381">
@@ -12249,7 +12249,7 @@
         <v>45958</v>
       </c>
       <c r="AV417">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="418">
@@ -13390,7 +13390,7 @@
         <v>45962</v>
       </c>
       <c r="AV458">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="459">
@@ -14462,7 +14462,7 @@
         <v>45954</v>
       </c>
       <c r="AV496">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="497">
@@ -15505,7 +15505,7 @@
         <v>45956</v>
       </c>
       <c r="AV533">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="534">
@@ -16692,7 +16692,7 @@
         <v>45964</v>
       </c>
       <c r="AV576">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="577">
@@ -17735,7 +17735,7 @@
         <v>45964</v>
       </c>
       <c r="AV613">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="614">

</xml_diff>